<commit_message>
data(padron): Genta Javier left by expulsion, not arrears
Operator correction of 26/08/2026 over the padron workbook, which is the
source of truth. An expelled member can never rejoin (Art. 5 inc. 2,
REG-04) and the reason is what the eligibility gate reads.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/padron_socios.xlsx
+++ b/datos/padron_socios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ciudadela\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE44531E-A51E-45ED-84D3-DB35B6781341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8377AA06-453A-4234-A704-803276BD82FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5A4086D6-E52A-46D6-AD6C-13484485911D}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="socios" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">socios!$A$1:$S$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">socios!$A$1:$S$279</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1723" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1723" uniqueCount="351">
   <si>
     <t>Castillo Nestor</t>
   </si>
@@ -1092,6 +1092,9 @@
   </si>
   <si>
     <t>martinrperez13@gmail.com</t>
+  </si>
+  <si>
+    <t>Expulsado</t>
   </si>
 </sst>
 </file>
@@ -3215,7 +3218,7 @@
         <v>45900</v>
       </c>
       <c r="S38" s="18" t="s">
-        <v>281</v>
+        <v>350</v>
       </c>
     </row>
     <row r="39" spans="1:19" s="22" customFormat="1" x14ac:dyDescent="0.2">
@@ -12585,7 +12588,7 @@
       <c r="S279" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S278" xr:uid="{1209BD55-AED0-4210-B3CC-BFEBD14B559A}"/>
+  <autoFilter ref="A1:S279" xr:uid="{1209BD55-AED0-4210-B3CC-BFEBD14B559A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S278">
     <sortCondition ref="A2:A278"/>
   </sortState>

</xml_diff>